<commit_message>
feat: mejorar import y rotadores de promociones
Genera slug y descripción automáticamente al importar desde Excel, agrega utilidades para corregir variantes de color de acero y actualiza las promos de home para rotar imágenes reales de collares y anillos.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/productos_template.xlsx
+++ b/productos_template.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\mary_mirari\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{127285E3-00F4-4BE5-ADF1-1B755D0370A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35564E61-FB6A-41AB-9937-B712667A7A7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="23">
   <si>
     <t>slug</t>
   </si>
@@ -57,58 +57,43 @@
     <t>extraImageUrls</t>
   </si>
   <si>
-    <t>DIJE</t>
-  </si>
-  <si>
-    <t>inserta descripcion ia</t>
+    <t>colors</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>true</t>
   </si>
   <si>
     <t>|</t>
   </si>
   <si>
-    <t>colors</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dsezvvmmt/image/upload/v1775527359/whatsapp-image-2026-03-18-at-1-44-50-pm-2-2a2c33ec82f8836e6b17738612780732-1024-1024_m2xg9t.webp</t>
-  </si>
-  <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dsezvvmmt/image/upload/v1775527518/whatsapp-image-2026-02-27-at-5-21-21-pm-14104535a834b0052317722254548817-480-0_zaglkt.webp</t>
-  </si>
-  <si>
-    <t>Dije colgante diamante color dorado por unidad</t>
-  </si>
-  <si>
-    <t>Dije por unidad serpiente color dorado</t>
-  </si>
-  <si>
-    <t>Dije tulipan dorado por unidad varios colores</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dsezvvmmt/image/upload/v1775527709/whatsapp-image-2026-03-18-at-1-44-27-pm-2e0c3c15b12764223e17738580245839-1024-1024_uwg0ok.webp</t>
-  </si>
-  <si>
-    <t>dorado rosa| dorado celeste | dorado blanco | dorado violeta</t>
-  </si>
-  <si>
-    <t>Dije zapatilla de tutbool acero quirúrgico</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dsezvvmmt/image/upload/v1775527861/img_5476-1f25e406e4e8d1c28217612209274230-1024-1024_vulmy8.webp</t>
-  </si>
-  <si>
-    <t>Boca | River</t>
-  </si>
-  <si>
-    <t>Dije por unidad luna+corazon</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dsezvvmmt/image/upload/v1775527972/whatsapp-image-2026-03-18-at-1-44-36-pm-3-a4244c079d0a48dfba17738647320031-1024-1024_y9ybus.webp</t>
-  </si>
-  <si>
-    <t>plateado | dorado</t>
+    <t>Anillo acero blanco</t>
+  </si>
+  <si>
+    <t>Anillo acero dorado</t>
+  </si>
+  <si>
+    <t>Anillo acero quirúrgico</t>
+  </si>
+  <si>
+    <t>anillo</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dsezvvmmt/image/upload/v1775547528/img_6109-3bdb61607617f0e1d917628008898155-1024-1024_dverhv.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dsezvvmmt/image/upload/v1775547528/img_6290-d61f992d92a003d6ac17631333557644-1024-1024_jv6pht.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dsezvvmmt/image/upload/v1775547529/img_6294-15511b0dfcb82f883417631356782259-1024-1024_kf7acp.webp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dsezvvmmt/image/upload/v1775547529/img_6082-b62dbd7384f03b0da917627893824026-1024-1024_upnv2e.webp</t>
+  </si>
+  <si>
+    <t>false</t>
   </si>
 </sst>
 </file>
@@ -117,7 +102,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -125,7 +110,7 @@
     </font>
     <font>
       <u/>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -154,15 +139,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -249,6 +234,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -283,6 +269,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -317,20 +304,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -452,15 +435,54 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -494,171 +516,184 @@
         <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
       <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2">
+        <v>5000</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
         <v>17</v>
       </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2">
-        <v>3000</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I2">
         <v>100</v>
       </c>
       <c r="J2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>5000</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3">
-        <v>2500</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>15</v>
       </c>
       <c r="I3">
         <v>100</v>
       </c>
       <c r="J3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
       </c>
       <c r="D4">
-        <v>3500</v>
+        <v>5000</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>20</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I4">
         <v>100</v>
       </c>
       <c r="J4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5">
+        <v>5000</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" t="s">
         <v>12</v>
-      </c>
-      <c r="K4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5">
-        <v>3500</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" t="s">
-        <v>15</v>
       </c>
       <c r="I5">
         <v>100</v>
       </c>
       <c r="J5" t="s">
-        <v>12</v>
-      </c>
-      <c r="K5" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6">
-        <v>2500</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6">
-        <v>100</v>
-      </c>
-      <c r="J6" t="s">
-        <v>12</v>
-      </c>
-      <c r="K6" t="s">
-        <v>27</v>
-      </c>
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E15" s="1"/>
+      <c r="J15" s="1"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E16" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{761BCD14-7132-49A0-812A-D744E34472D0}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{58F35B72-3AF0-437D-A331-4A947B9B9545}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{FACE5CF3-9596-484B-BFD7-1B1A71B12FB1}"/>
-    <hyperlink ref="E5" r:id="rId4" xr:uid="{D3E88C3B-4BB1-42F8-9F16-F0C41A3425D7}"/>
-    <hyperlink ref="E6" r:id="rId5" xr:uid="{5E243B76-1BC7-42F6-9E5C-537BC9D6397B}"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{E891CEDF-D15E-4536-8498-92307B3D6515}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{EE10EF77-CD55-4726-B134-8923D8BD9148}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{1922E614-199D-40E8-AE2D-D11F08AD257D}"/>
+    <hyperlink ref="E5" r:id="rId4" xr:uid="{C5B2853A-49C2-4CD8-9CB1-5BE0BD3E4933}"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:K1 A6 A2 C2 A3 C3 H2:J2 H3:J3 A4 C4 H4:J4 A5 C5 H5:J5" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>